<commit_message>
mail requirements 4 pointa
</commit_message>
<xml_diff>
--- a/card_status_gd.xlsx
+++ b/card_status_gd.xlsx
@@ -7,9 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Pending Cards(more than 30 days)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Abnormalities Cards" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Block" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ASSEMBLY (MK)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ASSEMBLY" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Crank" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Assembly-2 MK1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ASSEMBLY (HEAD SUB)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Piston Sub" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Check new" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Check" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pending Cards(more than 30 days)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Abnormalities Cards" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,14 +431,307 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>LINE</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>INPROGRESS</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>ASSEMBLY (MK)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Crank</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Assembly-2 MK1</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>ASSEMBLY (HEAD SUB)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Piston Sub</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Check new</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD Check LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CHK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>daily status id</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7327,7 +7629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7839,4 +8141,744 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD Block LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>another</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dummy 30 Jul 2024</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>achecld</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD ASSEMBLY (MK) LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TITM315</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>checking</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD ASSEMBLY LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TIBE323</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>checking</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD Crank LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OP150</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ccc</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OP105</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD Assembly-2 MK1 LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MK-5</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>checking</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD ASSEMBLY (HEAD SUB) LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TIAS334</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ceck</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD Piston Sub LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PS-3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>vvvvvv</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PS-2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>decison pending</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>white</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary of card raised in GD Check new LINE (last 30 days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP No.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Abnormality</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Pending Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CHKNEW</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>11 12 13</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>qqqqqqqqqqqqqqqwertyui</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>